<commit_message>
removed unused columns from averagePerDay_v5.xlsx
</commit_message>
<xml_diff>
--- a/data/averagePerDay_v5.xlsx
+++ b/data/averagePerDay_v5.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arshdeep\PycharmProjects\AI_DSA\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5951EB7F-D9E0-4B63-95D2-240CF1126018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28830" yWindow="840" windowWidth="10260" windowHeight="8595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="averagePerDay.csv" sheetId="1" r:id="rId4"/>
+    <sheet name="averagePerDay.csv" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="EQxmOlc032SZcQSny34i7TorEFhaSO80uld495fsR04="/>
@@ -16,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
   <si>
     <t>Hospital Name</t>
   </si>
@@ -36,9 +45,6 @@
     <t>discharges_per_hour</t>
   </si>
   <si>
-    <t>avg_beds_available</t>
-  </si>
-  <si>
     <t>Intensive Occupancy Rate</t>
   </si>
   <si>
@@ -55,9 +61,6 @@
   </si>
   <si>
     <t>occupancy rates</t>
-  </si>
-  <si>
-    <t>average_beds</t>
   </si>
   <si>
     <t>total_capacity</t>
@@ -101,15 +104,6 @@
     <t>[0.880713489409142, 0.87553457372952, 0.871146903637878]</t>
   </si>
   <si>
-    <t>[1.45309381237525, 5.86427145708583]</t>
-  </si>
-  <si>
-    <t>[0.5765765765765766, 0.281437125748503, 0.5508982035928144]</t>
-  </si>
-  <si>
-    <t>[0.1591591591591592, 0.6437125748502994, 0.9311377245508982]</t>
-  </si>
-  <si>
     <t>CHUQ</t>
   </si>
   <si>
@@ -136,15 +130,6 @@
     <t>[0.937241200828157, 0.93385765858690, 0.933277462609593]</t>
   </si>
   <si>
-    <t>[4.41167664670659, 1.89720558882236]</t>
-  </si>
-  <si>
-    <t>[0.5765765765765766, 0.2664670658682635, 0.781437125748503]</t>
-  </si>
-  <si>
-    <t>[0.4414414414414414, 0.8353293413173652, 0.9011976047904192]</t>
-  </si>
-  <si>
     <t>CHUS</t>
   </si>
   <si>
@@ -168,15 +153,6 @@
     <t>[0.864492753623188, 0.857039711191336, 0.851263537906137]</t>
   </si>
   <si>
-    <t>[1.73253493670659, 3.01596806882236]</t>
-  </si>
-  <si>
-    <t>[0.2372372372372372, 0.2335329341317365, 0.2664670658682635]</t>
-  </si>
-  <si>
-    <t>[0.1801801801801802, 0.311377245508982, 0.5958083832335329]</t>
-  </si>
-  <si>
     <t>CUSM</t>
   </si>
   <si>
@@ -198,15 +174,6 @@
     <t>[0.79180602006689, 0.789572341016384, 0.779852818661483]</t>
   </si>
   <si>
-    <t>[2.51097804670659, 7.51896207882236]</t>
-  </si>
-  <si>
-    <t>[0.6396396396396397, 0.07784431137724551, 0.6796407185628742]</t>
-  </si>
-  <si>
-    <t>[0.1591591591591592, 0.4640718562874251, 0.8832335329341318]</t>
-  </si>
-  <si>
     <t>HGJ</t>
   </si>
   <si>
@@ -228,15 +195,6 @@
     <t>[0.819266837169651, 0.812911446166914, 0.807390104056063]</t>
   </si>
   <si>
-    <t>[0.86626746670659, 7.13522954882236]</t>
-  </si>
-  <si>
-    <t>[0.4084084084084084, 0.2664670658682635, 0.3233532934131736]</t>
-  </si>
-  <si>
-    <t>[0.1291291291291291, 0.4341317365269461, 0.5568862275449101]</t>
-  </si>
-  <si>
     <t>HMR</t>
   </si>
   <si>
@@ -256,77 +214,64 @@
   </si>
   <si>
     <t>[0.83947628458498, 0.837725631768953, 0.823285198555957]</t>
-  </si>
-  <si>
-    <t>[0.84930139670659, 4.12924151882236]</t>
-  </si>
-  <si>
-    <t>[0.1501501501501502, 0.5449101796407185, 0.2844311377245509]</t>
-  </si>
-  <si>
-    <t>[0.2672672672672673, 0.3203592814371258, 0.4880239520958084]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="11">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="10">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
@@ -336,7 +281,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -346,7 +291,13 @@
     </fill>
   </fills>
   <borders count="4">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -360,8 +311,10 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -371,67 +324,60 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -621,35 +567,35 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <dimension ref="A1:Q1000"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="19.0"/>
-    <col customWidth="1" min="3" max="3" width="36.38"/>
-    <col customWidth="1" min="4" max="4" width="93.25"/>
-    <col customWidth="1" min="5" max="5" width="16.88"/>
-    <col customWidth="1" min="6" max="6" width="16.63"/>
-    <col customWidth="1" min="7" max="7" width="15.75"/>
-    <col customWidth="1" min="8" max="8" width="20.38"/>
-    <col customWidth="1" min="9" max="9" width="25.0"/>
-    <col customWidth="1" min="10" max="10" width="52.88"/>
-    <col customWidth="1" min="11" max="11" width="50.0"/>
-    <col customWidth="1" min="12" max="12" width="51.88"/>
-    <col customWidth="1" min="13" max="13" width="50.25"/>
-    <col customWidth="1" min="14" max="14" width="31.63"/>
-    <col customWidth="1" min="18" max="18" width="53.5"/>
-    <col customWidth="1" min="19" max="19" width="52.63"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="36.42578125" customWidth="1"/>
+    <col min="4" max="4" width="93.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="52.85546875" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="11" max="11" width="51.85546875" customWidth="1"/>
+    <col min="12" max="12" width="50.28515625" customWidth="1"/>
+    <col min="16" max="16" width="53.42578125" customWidth="1"/>
+    <col min="17" max="17" width="52.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" spans="1:17" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -668,409 +614,367 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="9" t="s">
+    </row>
+    <row r="2" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="1">
+        <v>6.5743512974051899E-2</v>
+      </c>
+      <c r="F2" s="1">
+        <v>7.3602794411177605E-2</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0.97061191599999996</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0.79380607299999995</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="10">
+        <v>65</v>
+      </c>
+      <c r="N2" s="6">
+        <v>30</v>
+      </c>
+      <c r="O2" s="6">
+        <v>35</v>
+      </c>
+      <c r="P2" s="11">
+        <v>5.8704662746578699E-2</v>
+      </c>
+      <c r="Q2" s="11">
+        <v>7.2250394106681298E-2</v>
+      </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="3" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5.6886227544910101E-2</v>
+      </c>
+      <c r="F3" s="1">
+        <v>7.3478043912175606E-2</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0.770323172</v>
+      </c>
+      <c r="H3" s="9">
+        <v>1.111893899</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" s="10">
+        <v>56</v>
+      </c>
+      <c r="N3" s="6">
+        <v>29</v>
+      </c>
+      <c r="O3" s="6">
+        <v>27</v>
+      </c>
+      <c r="P3" s="11">
+        <v>6.7686698674722295E-2</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>9.0748682814550993E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3.8672654690618702E-2</v>
+      </c>
+      <c r="F4" s="1">
+        <v>4.1791417165668601E-2</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0.91674215000000003</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0.81707930799999995</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" s="10">
         <v>20</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0.0657435129740519</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0.0736027944111776</v>
-      </c>
-      <c r="G2" s="1">
-        <v>5.57485029940119</v>
-      </c>
-      <c r="H2" s="12">
-        <v>0.970611916</v>
-      </c>
-      <c r="I2" s="12">
-        <v>0.793806073</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="1" t="s">
+      <c r="N4" s="6">
+        <v>8</v>
+      </c>
+      <c r="O4" s="6">
+        <v>12</v>
+      </c>
+      <c r="P4" s="11">
+        <v>3.07182182182167E-2</v>
+      </c>
+      <c r="Q4" s="11">
+        <v>4.5306908705112003E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="1">
+        <v>5.8008982035928101E-2</v>
+      </c>
+      <c r="F5" s="1">
+        <v>5.8507984031936099E-2</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0.93290133799999997</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0.64102564100000003</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M5" s="10">
+        <v>52</v>
+      </c>
+      <c r="N5" s="6">
         <v>26</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="O5" s="6">
+        <v>26</v>
+      </c>
+      <c r="P5" s="11">
+        <v>5.8213527899156299E-2</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>6.2769356182529698E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="1">
+        <v>4.6656686626746498E-2</v>
+      </c>
+      <c r="F6" s="1">
+        <v>4.7779441117764401E-2</v>
+      </c>
+      <c r="G6" s="9">
+        <v>1.0234644580000001</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0.66678744000000001</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" s="10">
+        <v>34</v>
+      </c>
+      <c r="N6" s="6">
+        <v>14</v>
+      </c>
+      <c r="O6" s="6">
+        <v>20</v>
+      </c>
+      <c r="P6" s="11">
+        <v>4.1592865320409997E-2</v>
+      </c>
+      <c r="Q6" s="11">
+        <v>4.6672795550041002E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="15.75" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="14">
-        <v>65.0</v>
-      </c>
-      <c r="P2" s="8">
-        <v>30.0</v>
-      </c>
-      <c r="Q2" s="8">
-        <v>35.0</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>29</v>
+      <c r="D7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="1">
+        <v>3.2559880239520902E-2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>3.73003992015968E-2</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0.990900856</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0.72992149799999995</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="10">
+        <v>20</v>
+      </c>
+      <c r="N7" s="6">
+        <v>8</v>
+      </c>
+      <c r="O7" s="6">
+        <v>12</v>
+      </c>
+      <c r="P7" s="11">
+        <v>4.0812144479809E-2</v>
+      </c>
+      <c r="Q7" s="11">
+        <v>4.4818770866675003E-2</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0.0568862275449101</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0.0734780439121756</v>
-      </c>
-      <c r="G3" s="1">
-        <v>4.40219560878243</v>
-      </c>
-      <c r="H3" s="12">
-        <v>0.770323172</v>
-      </c>
-      <c r="I3" s="12">
-        <v>1.111893899</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="O3" s="14">
-        <v>56.0</v>
-      </c>
-      <c r="P3" s="8">
-        <v>29.0</v>
-      </c>
-      <c r="Q3" s="8">
-        <v>27.0</v>
-      </c>
-      <c r="R3" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="S3" s="15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="1">
-        <v>0.0386726546906187</v>
-      </c>
-      <c r="F4" s="1">
-        <v>0.0417914171656686</v>
-      </c>
-      <c r="G4" s="1">
-        <v>4.27245508982035</v>
-      </c>
-      <c r="H4" s="12">
-        <v>0.91674215</v>
-      </c>
-      <c r="I4" s="12">
-        <v>0.817079308</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="O4" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="P4" s="8">
-        <v>8.0</v>
-      </c>
-      <c r="Q4" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="R4" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="S4" s="15" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0.0580089820359281</v>
-      </c>
-      <c r="F5" s="1">
-        <v>0.0585079840319361</v>
-      </c>
-      <c r="G5" s="1">
-        <v>9.37425149700598</v>
-      </c>
-      <c r="H5" s="12">
-        <v>0.932901338</v>
-      </c>
-      <c r="I5" s="12">
-        <v>0.641025641</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" s="14">
-        <v>52.0</v>
-      </c>
-      <c r="P5" s="8">
-        <v>26.0</v>
-      </c>
-      <c r="Q5" s="8">
-        <v>26.0</v>
-      </c>
-      <c r="R5" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="S5" s="15" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0.0466566866267465</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0.0477794411177644</v>
-      </c>
-      <c r="G6" s="1">
-        <v>7.0878243512974</v>
-      </c>
-      <c r="H6" s="12">
-        <v>1.023464458</v>
-      </c>
-      <c r="I6" s="12">
-        <v>0.66678744</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="N6" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="O6" s="14">
-        <v>34.0</v>
-      </c>
-      <c r="P6" s="8">
-        <v>14.0</v>
-      </c>
-      <c r="Q6" s="8">
-        <v>20.0</v>
-      </c>
-      <c r="R6" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.0325598802395209</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0.0373003992015968</v>
-      </c>
-      <c r="G7" s="1">
-        <v>4.08882235528942</v>
-      </c>
-      <c r="H7" s="12">
-        <v>0.990900856</v>
-      </c>
-      <c r="I7" s="12">
-        <v>0.729921498</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="N7" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="O7" s="14">
-        <v>20.0</v>
-      </c>
-      <c r="P7" s="8">
-        <v>8.0</v>
-      </c>
-      <c r="Q7" s="8">
-        <v>12.0</v>
-      </c>
-      <c r="R7" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="S7" s="15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1"/>
-    <row r="9" ht="15.75" customHeight="1"/>
-    <row r="10" ht="15.75" customHeight="1"/>
-    <row r="11" ht="15.75" customHeight="1"/>
-    <row r="12" ht="15.75" customHeight="1"/>
-    <row r="13" ht="15.75" customHeight="1"/>
-    <row r="14" ht="15.75" customHeight="1"/>
-    <row r="15" ht="15.75" customHeight="1"/>
-    <row r="16" ht="15.75" customHeight="1"/>
+    <row r="8" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="9" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="10" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="11" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="12" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="13" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="14" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="15" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="16" spans="1:17" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -2056,9 +1960,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.0" footer="0.0" header="0.0" left="0.0" right="0.0" top="0.0"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added patients transferred from another hospital
</commit_message>
<xml_diff>
--- a/data/averagePerDay_v5.xlsx
+++ b/data/averagePerDay_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arshdeep\PycharmProjects\AI_DSA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5951EB7F-D9E0-4B63-95D2-240CF1126018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F2A646-40C7-497C-9A96-A4245C8502F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28830" yWindow="840" windowWidth="10260" windowHeight="8595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34545" yWindow="1665" windowWidth="21270" windowHeight="13710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="averagePerDay.csv" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="62">
   <si>
     <t>Hospital Name</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>[0.83947628458498, 0.837725631768953, 0.823285198555957]</t>
+  </si>
+  <si>
+    <t>transfer_percentage</t>
   </si>
 </sst>
 </file>
@@ -577,7 +580,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q1000"/>
+  <dimension ref="A1:R1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -595,7 +598,7 @@
     <col min="17" max="17" width="52.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" customHeight="1">
+    <row r="1" spans="1:18" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -647,8 +650,11 @@
       <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="R1" t="s">
+        <v>61</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" customHeight="1">
+    <row r="2" spans="1:18" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -700,8 +706,11 @@
       <c r="Q2" s="11">
         <v>7.2250394106681298E-2</v>
       </c>
+      <c r="R2">
+        <v>39.964975796942753</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" customHeight="1">
+    <row r="3" spans="1:18" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -753,8 +762,11 @@
       <c r="Q3" s="11">
         <v>9.0748682814550993E-2</v>
       </c>
+      <c r="R3">
+        <v>2.9628276640243301</v>
+      </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" customHeight="1">
+    <row r="4" spans="1:18" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
@@ -806,8 +818,11 @@
       <c r="Q4" s="11">
         <v>4.5306908705112003E-2</v>
       </c>
+      <c r="R4">
+        <v>7.5028842238327584</v>
+      </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" customHeight="1">
+    <row r="5" spans="1:18" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>40</v>
       </c>
@@ -859,8 +874,11 @@
       <c r="Q5" s="11">
         <v>6.2769356182529698E-2</v>
       </c>
+      <c r="R5">
+        <v>60.320736263752188</v>
+      </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" customHeight="1">
+    <row r="6" spans="1:18" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>47</v>
       </c>
@@ -912,8 +930,11 @@
       <c r="Q6" s="11">
         <v>4.6672795550041002E-2</v>
       </c>
+      <c r="R6">
+        <v>14.982732330933359</v>
+      </c>
     </row>
-    <row r="7" spans="1:17" ht="15.75" customHeight="1">
+    <row r="7" spans="1:18" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>54</v>
       </c>
@@ -965,16 +986,19 @@
       <c r="Q7" s="11">
         <v>4.4818770866675003E-2</v>
       </c>
+      <c r="R7">
+        <v>9.7269662872853306</v>
+      </c>
     </row>
-    <row r="8" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="10" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="11" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:17" ht="15.75" customHeight="1"/>
+    <row r="8" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="9" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="10" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="11" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="12" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="13" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="14" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="15" spans="1:18" ht="15.75" customHeight="1"/>
+    <row r="16" spans="1:18" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Changed the admit patient function temporarily because more patients were being admitted than capacity
</commit_message>
<xml_diff>
--- a/data/averagePerDay_v5.xlsx
+++ b/data/averagePerDay_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arshdeep\PycharmProjects\AI_DSA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F2A646-40C7-497C-9A96-A4245C8502F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514357D2-E682-4776-AC25-0154AE5B6417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34545" yWindow="1665" windowWidth="21270" windowHeight="13710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22395" yWindow="960" windowWidth="20370" windowHeight="12555" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="averagePerDay.csv" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t>[0.155688623, 0.592814371, 1.017964072]</t>
   </si>
   <si>
-    <t>[5.4251497005988, 6, 5.29940119760479]</t>
-  </si>
-  <si>
     <t>[0.880713489409142, 0.87553457372952, 0.871146903637878]</t>
   </si>
   <si>
@@ -124,9 +121,6 @@
     <t>[0.284431138, 0.679640719, 0.799401198]</t>
   </si>
   <si>
-    <t>[4.4191616766467, 4.65868263473053, 4.12874251497006]</t>
-  </si>
-  <si>
     <t>[0.937241200828157, 0.93385765858690, 0.933277462609593]</t>
   </si>
   <si>
@@ -147,9 +141,6 @@
     <t>[0.107784431, 0.311377246, 0.583832335]</t>
   </si>
   <si>
-    <t>[4.19161676646706, 4.54790419161676, 4.07784431137724 ]</t>
-  </si>
-  <si>
     <t>[0.864492753623188, 0.857039711191336, 0.851263537906137]</t>
   </si>
   <si>
@@ -168,9 +159,6 @@
     <t>[0.146706587, 0.362275449, 0.895209581]</t>
   </si>
   <si>
-    <t>[9.15868263473053, 9.76646706586826, 9.19760479041916 ]</t>
-  </si>
-  <si>
     <t>[0.79180602006689, 0.789572341016384, 0.779852818661483]</t>
   </si>
   <si>
@@ -189,9 +177,6 @@
     <t>[0.119760479, 0.464071856, 0.562874251]</t>
   </si>
   <si>
-    <t>[7.09281437125748, 7.2814371257485, 6.88922155688622]</t>
-  </si>
-  <si>
     <t>[0.819266837169651, 0.812911446166914, 0.807390104056063]</t>
   </si>
   <si>
@@ -210,13 +195,28 @@
     <t>[0.116766467, 0.371257485, 0.407185629]</t>
   </si>
   <si>
-    <t>[4.07185628742515, 4.20958083832335, 3.98502994011976 ]</t>
-  </si>
-  <si>
     <t>[0.83947628458498, 0.837725631768953, 0.823285198555957]</t>
   </si>
   <si>
     <t>transfer_percentage</t>
+  </si>
+  <si>
+    <t>[5.4251497005988, 6]</t>
+  </si>
+  <si>
+    <t>[4.4191616766467, 4.65868263473053]</t>
+  </si>
+  <si>
+    <t>[4.19161676646706, 4.54790419161676 ]</t>
+  </si>
+  <si>
+    <t>[9.15868263473053, 9.76646706586826 ]</t>
+  </si>
+  <si>
+    <t>[7.09281437125748, 7.2814371257485]</t>
+  </si>
+  <si>
+    <t>[4.07185628742515, 4.20958083832335 ]</t>
   </si>
 </sst>
 </file>
@@ -651,7 +651,7 @@
         <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="15.75" customHeight="1">
@@ -686,10 +686,10 @@
         <v>22</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="M2" s="10">
         <v>65</v>
@@ -712,16 +712,16 @@
     </row>
     <row r="3" spans="1:18" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="12" t="s">
         <v>27</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>28</v>
       </c>
       <c r="E3" s="1">
         <v>5.6886227544910101E-2</v>
@@ -736,16 +736,16 @@
         <v>1.111893899</v>
       </c>
       <c r="I3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="M3" s="10">
         <v>56</v>
@@ -768,16 +768,16 @@
     </row>
     <row r="4" spans="1:18" ht="15.75" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="E4" s="1">
         <v>3.8672654690618702E-2</v>
@@ -792,16 +792,16 @@
         <v>0.81707930799999995</v>
       </c>
       <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="L4" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="M4" s="10">
         <v>20</v>
@@ -824,16 +824,16 @@
     </row>
     <row r="5" spans="1:18" ht="15.75" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1">
         <v>5.8008982035928101E-2</v>
@@ -848,16 +848,16 @@
         <v>0.64102564100000003</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="M5" s="10">
         <v>52</v>
@@ -880,16 +880,16 @@
     </row>
     <row r="6" spans="1:18" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E6" s="1">
         <v>4.6656686626746498E-2</v>
@@ -904,16 +904,16 @@
         <v>0.66678744000000001</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="M6" s="10">
         <v>34</v>
@@ -936,16 +936,16 @@
     </row>
     <row r="7" spans="1:18" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E7" s="1">
         <v>3.2559880239520902E-2</v>
@@ -960,16 +960,16 @@
         <v>0.72992149799999995</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="M7" s="10">
         <v>20</v>

</xml_diff>

<commit_message>
Add Indigenous bool attribute to the patient
</commit_message>
<xml_diff>
--- a/data/averagePerDay_v5.xlsx
+++ b/data/averagePerDay_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dohee\Desktop\Korah\Simulator2\AI_DSA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0020F91-04E8-4FCD-BBAB-FA8510FBA6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80A7650-4985-4BC0-BF0F-90141C6B9C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2250" yWindow="90" windowWidth="25410" windowHeight="20790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24360" yWindow="380" windowWidth="25410" windowHeight="20790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="averagePerDay.csv" sheetId="1" r:id="rId1"/>
@@ -859,11 +859,11 @@
       <c r="R2" s="13">
         <v>35</v>
       </c>
-      <c r="S2" s="14">
-        <v>5.8704662746578699E-2</v>
-      </c>
-      <c r="T2" s="14">
-        <v>7.2250394106681298E-2</v>
+      <c r="S2">
+        <v>7.5489243595431396E-2</v>
+      </c>
+      <c r="T2">
+        <v>7.7641250978343804E-2</v>
       </c>
       <c r="U2" s="14">
         <v>39.964975796942753</v>
@@ -924,11 +924,11 @@
       <c r="R3" s="13">
         <v>27</v>
       </c>
-      <c r="S3" s="14">
-        <v>0.04</v>
-      </c>
-      <c r="T3" s="14">
-        <v>0.03</v>
+      <c r="S3">
+        <v>3.03261623969543E-2</v>
+      </c>
+      <c r="T3">
+        <v>5.54580364131027E-2</v>
       </c>
       <c r="U3" s="14">
         <v>2.9628276640243301</v>
@@ -989,11 +989,11 @@
       <c r="R4" s="13">
         <v>12</v>
       </c>
-      <c r="S4" s="14">
-        <v>0.02</v>
-      </c>
-      <c r="T4" s="14">
-        <v>0.01</v>
+      <c r="S4">
+        <v>2.51630811984771E-2</v>
+      </c>
+      <c r="T4">
+        <v>2.21832145652411E-2</v>
       </c>
       <c r="U4" s="14">
         <v>7.5028842238327584</v>
@@ -1054,11 +1054,11 @@
       <c r="R5" s="13">
         <v>26</v>
       </c>
-      <c r="S5" s="14">
-        <v>5.8213527899156299E-2</v>
-      </c>
-      <c r="T5" s="14">
-        <v>0.04</v>
+      <c r="S5">
+        <v>7.5489243595431396E-2</v>
+      </c>
+      <c r="T5">
+        <v>6.6549643695723304E-2</v>
       </c>
       <c r="U5" s="14">
         <v>60.320736263752188</v>
@@ -1119,11 +1119,11 @@
       <c r="R6" s="13">
         <v>20</v>
       </c>
-      <c r="S6" s="14">
-        <v>4.1592865320409997E-2</v>
-      </c>
-      <c r="T6" s="14">
-        <v>0.03</v>
+      <c r="S6">
+        <v>5.0326162396954303E-2</v>
+      </c>
+      <c r="T6">
+        <v>5.54580364131027E-2</v>
       </c>
       <c r="U6" s="14">
         <v>14.982732330933359</v>
@@ -1184,11 +1184,11 @@
       <c r="R7" s="13">
         <v>12</v>
       </c>
-      <c r="S7" s="14">
-        <v>0.09</v>
-      </c>
-      <c r="T7" s="14">
-        <v>0.05</v>
+      <c r="S7">
+        <v>0.113233865393147</v>
+      </c>
+      <c r="T7">
+        <v>8.8732858260964401E-2</v>
       </c>
       <c r="U7" s="14">
         <v>9.7269662872853306</v>

</xml_diff>

<commit_message>
Adjust the discharged rate and condition occupancy rate for each bed type
</commit_message>
<xml_diff>
--- a/data/averagePerDay_v5.xlsx
+++ b/data/averagePerDay_v5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dohee\Desktop\Korah\Simulator2\AI_DSA\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dohee\Desktop\Korah\AI_DSA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A80A7650-4985-4BC0-BF0F-90141C6B9C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91624CDB-86FA-43E6-B0B2-E74C2285CD5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24360" yWindow="380" windowWidth="25410" windowHeight="20790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="averagePerDay.csv" sheetId="1" r:id="rId1"/>
@@ -717,29 +717,30 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:U1000"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="93.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="56.7265625" style="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.54296875" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.453125" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.1328125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="93.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.86328125" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="56.73046875" style="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.59765625" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.3984375" style="16" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25" style="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="52.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="52.86328125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="51.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="50.26953125" bestFit="1" customWidth="1"/>
-    <col min="16" max="18" width="14.1796875" style="17" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="53.453125" style="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="52.54296875" style="16" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.1796875" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="51.86328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="50.265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="18" width="14.1328125" style="17" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="53.3984375" style="16" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="52.59765625" style="16" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.1328125" style="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="19.5" customHeight="1">
+    <row r="1" spans="1:21" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -859,11 +860,11 @@
       <c r="R2" s="13">
         <v>35</v>
       </c>
-      <c r="S2">
-        <v>7.5489243595431396E-2</v>
-      </c>
-      <c r="T2">
-        <v>7.7641250978343804E-2</v>
+      <c r="S2" s="14">
+        <v>5.8704662746578699E-2</v>
+      </c>
+      <c r="T2" s="14">
+        <v>7.2250394106681298E-2</v>
       </c>
       <c r="U2" s="14">
         <v>39.964975796942753</v>
@@ -924,11 +925,11 @@
       <c r="R3" s="13">
         <v>27</v>
       </c>
-      <c r="S3">
-        <v>3.03261623969543E-2</v>
-      </c>
-      <c r="T3">
-        <v>5.54580364131027E-2</v>
+      <c r="S3" s="14">
+        <v>3.3843349330000001E-2</v>
+      </c>
+      <c r="T3" s="14">
+        <v>4.5374341399999997E-2</v>
       </c>
       <c r="U3" s="14">
         <v>2.9628276640243301</v>
@@ -989,11 +990,11 @@
       <c r="R4" s="13">
         <v>12</v>
       </c>
-      <c r="S4">
-        <v>2.51630811984771E-2</v>
-      </c>
-      <c r="T4">
-        <v>2.21832145652411E-2</v>
+      <c r="S4" s="14">
+        <v>1.5359109100000001E-2</v>
+      </c>
+      <c r="T4" s="14">
+        <v>1.5359109100000001E-2</v>
       </c>
       <c r="U4" s="14">
         <v>7.5028842238327584</v>
@@ -1054,11 +1055,11 @@
       <c r="R5" s="13">
         <v>26</v>
       </c>
-      <c r="S5">
-        <v>7.5489243595431396E-2</v>
-      </c>
-      <c r="T5">
-        <v>6.6549643695723304E-2</v>
+      <c r="S5" s="14">
+        <v>5.8213527899156299E-2</v>
+      </c>
+      <c r="T5" s="14">
+        <v>3.138467809E-2</v>
       </c>
       <c r="U5" s="14">
         <v>60.320736263752188</v>
@@ -1119,11 +1120,11 @@
       <c r="R6" s="13">
         <v>20</v>
       </c>
-      <c r="S6">
-        <v>5.0326162396954303E-2</v>
-      </c>
-      <c r="T6">
-        <v>5.54580364131027E-2</v>
+      <c r="S6" s="14">
+        <v>4.1592865320409997E-2</v>
+      </c>
+      <c r="T6" s="14">
+        <v>2.333639777E-2</v>
       </c>
       <c r="U6" s="14">
         <v>14.982732330933359</v>
@@ -1184,27 +1185,27 @@
       <c r="R7" s="13">
         <v>12</v>
       </c>
-      <c r="S7">
-        <v>0.113233865393147</v>
-      </c>
-      <c r="T7">
-        <v>8.8732858260964401E-2</v>
+      <c r="S7" s="14">
+        <v>4.0812144479809E-2</v>
+      </c>
+      <c r="T7" s="14">
+        <v>4.4818770866675003E-2</v>
       </c>
       <c r="U7" s="14">
         <v>9.7269662872853306</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="9" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="10" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="11" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="12" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="13" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="14" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="15" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="16" spans="1:21" ht="18.75" customHeight="1"/>
-    <row r="17" ht="18.75" customHeight="1"/>
-    <row r="18" ht="18.75" customHeight="1"/>
+    <row r="8" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="9" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="10" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="11" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="12" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="13" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="14" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="15" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="16" spans="1:21" ht="19.5" customHeight="1"/>
+    <row r="17" ht="19.5" customHeight="1"/>
+    <row r="18" ht="19.5" customHeight="1"/>
     <row r="19" ht="18.75" customHeight="1"/>
     <row r="20" ht="18.75" customHeight="1"/>
     <row r="21" ht="18.75" customHeight="1"/>

</xml_diff>